<commit_message>
Folha nova da usinagem: códigos 1–10 (9 set-up, 10 ferramenta), A4 em PDF e orientação A3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019Px7p5mhzWYWbE6aV5W89g
</commit_message>
<xml_diff>
--- a/docs/folha-modelo/diario-de-bordo.xlsx
+++ b/docs/folha-modelo/diario-de-bordo.xlsx
@@ -2950,7 +2950,7 @@
       <c r="I18" s="17" t="inlineStr">
         <is>
           <t>MOTIVO
-(código 1–9)</t>
+(código 1–10)</t>
         </is>
       </c>
       <c r="J18" s="38" t="n"/>
@@ -3597,7 +3597,25 @@
               <color rgb="FF111111"/>
               <sz val="9"/>
             </rPr>
-            <t xml:space="preserve">  Troca de peça</t>
+            <t xml:space="preserve">  Troca de peça
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="9"/>
+            </rPr>
+            <t>5</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Falta de peça</t>
           </r>
         </is>
       </c>
@@ -3612,24 +3630,6 @@
               <color rgb="FF111111"/>
               <sz val="9"/>
             </rPr>
-            <t>5</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="9"/>
-            </rPr>
-            <t xml:space="preserve">  Falta de peça
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="9"/>
-            </rPr>
             <t>6</t>
           </r>
           <r>
@@ -3692,7 +3692,25 @@
               <color rgb="FF111111"/>
               <sz val="9"/>
             </rPr>
-            <t xml:space="preserve">  Set-up</t>
+            <t xml:space="preserve">  Set-up
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="9"/>
+            </rPr>
+            <t>10</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Ferramenta</t>
           </r>
         </is>
       </c>
@@ -3732,7 +3750,7 @@
               <color rgb="FF111111"/>
               <sz val="8.5"/>
             </rPr>
-            <t xml:space="preserve">Nº da peça 1 · 14:30–15:30 · motivo 9 (set-up)
+            <t xml:space="preserve">Nº da peça 1 · 14:30–15:30 · motivo 10 (troca de inserto)
 </t>
           </r>
           <r>

</xml_diff>

<commit_message>
Folhas A4 (robô e usinagem) ocupam a página inteira: colunas mais largas e margens menores
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019Px7p5mhzWYWbE6aV5W89g
</commit_message>
<xml_diff>
--- a/docs/folha-modelo/diario-de-bordo.xlsx
+++ b/docs/folha-modelo/diario-de-bordo.xlsx
@@ -822,21 +822,25 @@
   <dimension ref="A1:S38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="7.42578125" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="6.5703125" customWidth="1" min="6" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="6.5703125" customWidth="1" min="9" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="6.5703125" customWidth="1" min="12" max="13"/>
-    <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="6.5703125" customWidth="1" min="15" max="16"/>
-    <col width="9.42578125" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="6.05" customWidth="1" min="1" max="1"/>
+    <col width="8.99" customWidth="1" min="2" max="2"/>
+    <col width="19.36" customWidth="1" min="3" max="3"/>
+    <col width="16.94" customWidth="1" min="4" max="4"/>
+    <col width="8.470000000000001" customWidth="1" min="5" max="5"/>
+    <col width="7.95" customWidth="1" min="6" max="7"/>
+    <col width="15.73" customWidth="1" min="7" max="7"/>
+    <col width="8.470000000000001" customWidth="1" min="8" max="8"/>
+    <col width="7.95" customWidth="1" min="9" max="10"/>
+    <col width="15.73" customWidth="1" min="10" max="10"/>
+    <col width="8.470000000000001" customWidth="1" min="11" max="11"/>
+    <col width="7.95" customWidth="1" min="12" max="13"/>
+    <col width="15.73" customWidth="1" min="13" max="13"/>
+    <col width="8.470000000000001" customWidth="1" min="14" max="14"/>
+    <col width="7.95" customWidth="1" min="15" max="16"/>
+    <col width="15.73" customWidth="1" min="16" max="16"/>
+    <col width="11.41" customWidth="1" min="17" max="17"/>
+    <col width="12.1" customWidth="1" min="18" max="18"/>
+    <col width="22.99" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -2358,7 +2362,7 @@
     <mergeCell ref="C5:C6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0" footer="0"/>
+  <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0" footer="0"/>
   <pageSetup orientation="landscape" paperSize="9" scale="77"/>
 </worksheet>
 </file>
@@ -2372,21 +2376,25 @@
   <dimension ref="A1:S38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="7.42578125" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="6.5703125" customWidth="1" min="6" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="6.5703125" customWidth="1" min="9" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="6.5703125" customWidth="1" min="12" max="13"/>
-    <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="6.5703125" customWidth="1" min="15" max="16"/>
-    <col width="9.42578125" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="6.05" customWidth="1" min="1" max="1"/>
+    <col width="8.99" customWidth="1" min="2" max="2"/>
+    <col width="19.36" customWidth="1" min="3" max="3"/>
+    <col width="16.94" customWidth="1" min="4" max="4"/>
+    <col width="8.470000000000001" customWidth="1" min="5" max="5"/>
+    <col width="7.95" customWidth="1" min="6" max="7"/>
+    <col width="15.73" customWidth="1" min="7" max="7"/>
+    <col width="8.470000000000001" customWidth="1" min="8" max="8"/>
+    <col width="7.95" customWidth="1" min="9" max="10"/>
+    <col width="15.73" customWidth="1" min="10" max="10"/>
+    <col width="8.470000000000001" customWidth="1" min="11" max="11"/>
+    <col width="7.95" customWidth="1" min="12" max="13"/>
+    <col width="15.73" customWidth="1" min="13" max="13"/>
+    <col width="8.470000000000001" customWidth="1" min="14" max="14"/>
+    <col width="7.95" customWidth="1" min="15" max="16"/>
+    <col width="15.73" customWidth="1" min="16" max="16"/>
+    <col width="11.41" customWidth="1" min="17" max="17"/>
+    <col width="12.1" customWidth="1" min="18" max="18"/>
+    <col width="22.99" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -3944,7 +3952,7 @@
     <mergeCell ref="C5:C6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0" footer="0"/>
+  <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0" footer="0"/>
   <pageSetup orientation="landscape" paperSize="9" scale="77"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Folhas A4: letras maiores nos quadros Como preencher, Códigos e Exemplo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019Px7p5mhzWYWbE6aV5W89g
</commit_message>
<xml_diff>
--- a/docs/folha-modelo/diario-de-bordo.xlsx
+++ b/docs/folha-modelo/diario-de-bordo.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -140,6 +140,14 @@
       <family val="2"/>
       <b val="1"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10.5"/>
     </font>
   </fonts>
   <fills count="6">
@@ -342,7 +350,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -454,6 +462,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1687,13 +1701,13 @@
       <c r="S31" s="37" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="23" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="8.5"/>
+      <c r="A32" s="45" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">1. </t>
           </r>
@@ -1702,7 +1716,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Uma linha = uma peça.</t>
           </r>
@@ -1710,7 +1724,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> Começou peça nova? Linha nova.
 </t>
@@ -1719,7 +1733,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">2. </t>
           </r>
@@ -1728,7 +1742,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Trecho</t>
           </r>
@@ -1736,7 +1750,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> = tempo produzindo, </t>
           </r>
@@ -1745,7 +1759,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>sem parada no meio</t>
           </r>
@@ -1753,7 +1767,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">. Parou a máquina? </t>
           </r>
@@ -1762,7 +1776,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Feche o trecho</t>
           </r>
@@ -1770,7 +1784,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> (FIM).
 </t>
@@ -1779,7 +1793,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">3. Anote a parada no </t>
           </r>
@@ -1788,7 +1802,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>quadro 2</t>
           </r>
@@ -1796,7 +1810,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">, com o </t>
           </r>
@@ -1805,7 +1819,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Nº da peça</t>
           </r>
@@ -1813,7 +1827,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> e o código do motivo.
 </t>
@@ -1822,7 +1836,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">4. Voltou a produzir a mesma peça? Use o </t>
           </r>
@@ -1831,7 +1845,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>próximo trecho da mesma linha</t>
           </r>
@@ -1839,7 +1853,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">.
 </t>
@@ -1848,7 +1862,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">5. Troca de turno no meio da peça: o próximo operador usa o próximo trecho, com a chapa dele.
 </t>
@@ -1857,7 +1871,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">6. </t>
           </r>
@@ -1866,7 +1880,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Peça pronta?</t>
           </r>
@@ -1874,7 +1888,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> Escreva em </t>
           </r>
@@ -1883,7 +1897,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>PRONTA</t>
           </r>
@@ -1891,7 +1905,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> o </t>
           </r>
@@ -1900,7 +1914,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>turno que finalizou</t>
           </r>
@@ -1908,7 +1922,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> (1, 2 ou 3). Não terminou? Deixe em branco e continue na próxima folha.
 </t>
@@ -1917,7 +1931,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">7. </t>
           </r>
@@ -1926,7 +1940,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Mais de 4 trechos na mesma peça?</t>
           </r>
@@ -1934,7 +1948,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> Continue na </t>
           </r>
@@ -1943,7 +1957,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>linha de baixo</t>
           </r>
@@ -1951,7 +1965,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">, com a mesma peça, e escreva em </t>
           </r>
@@ -1960,7 +1974,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>CONTINUA A PEÇA Nº</t>
           </r>
@@ -1968,7 +1982,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> o número da linha de cima. O turno em PRONTA vai só na última linha.</t>
           </r>
@@ -1987,7 +2001,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>1</t>
           </r>
@@ -1995,7 +2009,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Mecânica
 </t>
@@ -2005,7 +2019,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>2</t>
           </r>
@@ -2013,7 +2027,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Elétrica
 </t>
@@ -2023,7 +2037,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>3</t>
           </r>
@@ -2031,7 +2045,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Manutenção preventiva
 </t>
@@ -2041,7 +2055,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>4</t>
           </r>
@@ -2049,7 +2063,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Troca de peça</t>
           </r>
@@ -2064,7 +2078,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>5</t>
           </r>
@@ -2072,7 +2086,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Falta de peça
 </t>
@@ -2082,7 +2096,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>6</t>
           </r>
@@ -2090,7 +2104,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Refeição
 </t>
@@ -2100,7 +2114,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>7</t>
           </r>
@@ -2108,7 +2122,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Tyorei
 </t>
@@ -2118,7 +2132,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>8</t>
           </r>
@@ -2126,21 +2140,21 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Outros (descreva)</t>
           </r>
         </is>
       </c>
       <c r="L32" s="36" t="n"/>
-      <c r="M32" s="23" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="8.5"/>
+      <c r="M32" s="46" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">Quadro 1 (peça 1): </t>
           </r>
@@ -2148,7 +2162,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">VIGA · D51 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · Pronta: 1
 </t>
@@ -2158,7 +2172,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">Quadro 2: </t>
           </r>
@@ -2166,7 +2180,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">Nº da peça 1 · 14:30–15:30 · motivo 5 (falta de peça)
 </t>
@@ -2176,7 +2190,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">Certo: </t>
           </r>
@@ -2184,7 +2198,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">3 h de produção + 1 h parada = 4 h.
 </t>
@@ -2194,7 +2208,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">Errado: </t>
           </r>
@@ -2202,7 +2216,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>um trecho 13:00–17:00 com a parada dentro dele (a hora parada conta duas vezes).</t>
           </r>
@@ -3241,13 +3255,13 @@
       <c r="S31" s="37" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="23" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="8.5"/>
+      <c r="A32" s="45" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">1. </t>
           </r>
@@ -3256,7 +3270,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Uma linha = uma peça.</t>
           </r>
@@ -3264,7 +3278,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> Começou peça nova? Linha nova.
 </t>
@@ -3273,7 +3287,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">2. </t>
           </r>
@@ -3282,7 +3296,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Trecho</t>
           </r>
@@ -3290,7 +3304,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> = tempo produzindo, </t>
           </r>
@@ -3299,7 +3313,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>sem parada no meio</t>
           </r>
@@ -3307,7 +3321,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">. Parou a máquina? </t>
           </r>
@@ -3316,7 +3330,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Feche o trecho</t>
           </r>
@@ -3324,7 +3338,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> (FIM).
 </t>
@@ -3333,7 +3347,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">3. Anote a parada no </t>
           </r>
@@ -3342,7 +3356,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>quadro 2</t>
           </r>
@@ -3350,7 +3364,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">, com o </t>
           </r>
@@ -3359,7 +3373,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Nº da peça</t>
           </r>
@@ -3367,7 +3381,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> e o código do motivo.
 </t>
@@ -3376,7 +3390,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">4. Voltou a produzir a mesma peça? Use o </t>
           </r>
@@ -3385,7 +3399,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>próximo trecho da mesma linha</t>
           </r>
@@ -3393,7 +3407,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">.
 </t>
@@ -3402,7 +3416,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">5. Troca de turno no meio da peça: o próximo operador usa o próximo trecho, com a chapa dele.
 </t>
@@ -3411,7 +3425,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">6. </t>
           </r>
@@ -3420,7 +3434,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Peça pronta?</t>
           </r>
@@ -3428,7 +3442,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> Escreva em </t>
           </r>
@@ -3437,7 +3451,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>PRONTA</t>
           </r>
@@ -3445,7 +3459,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> o </t>
           </r>
@@ -3454,7 +3468,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>turno que finalizou</t>
           </r>
@@ -3462,7 +3476,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> (1, 2 ou 3). Não terminou? Deixe em branco e continue na próxima folha.
 </t>
@@ -3471,7 +3485,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">7. </t>
           </r>
@@ -3480,7 +3494,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>Mais de 4 trechos na mesma peça?</t>
           </r>
@@ -3488,7 +3502,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> Continue na </t>
           </r>
@@ -3497,7 +3511,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>linha de baixo</t>
           </r>
@@ -3505,7 +3519,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve">, com a mesma peça, e escreva em </t>
           </r>
@@ -3514,7 +3528,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t>CONTINUA A PEÇA Nº</t>
           </r>
@@ -3522,7 +3536,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="9.5"/>
             </rPr>
             <t xml:space="preserve"> o número da linha de cima. O turno em PRONTA vai só na última linha.</t>
           </r>
@@ -3541,7 +3555,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>1</t>
           </r>
@@ -3549,7 +3563,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Mecânica
 </t>
@@ -3559,7 +3573,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>2</t>
           </r>
@@ -3567,7 +3581,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Elétrica
 </t>
@@ -3577,7 +3591,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>3</t>
           </r>
@@ -3585,7 +3599,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Manutenção preventiva
 </t>
@@ -3595,7 +3609,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>4</t>
           </r>
@@ -3603,7 +3617,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Troca de peça
 </t>
@@ -3613,7 +3627,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>5</t>
           </r>
@@ -3621,7 +3635,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Falta de peça</t>
           </r>
@@ -3636,7 +3650,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>6</t>
           </r>
@@ -3644,7 +3658,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Refeição
 </t>
@@ -3654,7 +3668,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>7</t>
           </r>
@@ -3662,7 +3676,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Tyorei
 </t>
@@ -3672,7 +3686,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>8</t>
           </r>
@@ -3680,7 +3694,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Outros (descreva)
 </t>
@@ -3690,7 +3704,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>9</t>
           </r>
@@ -3698,7 +3712,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Set-up
 </t>
@@ -3708,7 +3722,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t>10</t>
           </r>
@@ -3716,21 +3730,21 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">  Ferramenta</t>
           </r>
         </is>
       </c>
       <c r="L32" s="36" t="n"/>
-      <c r="M32" s="23" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="8.5"/>
+      <c r="M32" s="46" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">Quadro 1 (peça 1): </t>
           </r>
@@ -3738,7 +3752,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">MESA · D61 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · Pronta: 1
 </t>
@@ -3748,7 +3762,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">Quadro 2: </t>
           </r>
@@ -3756,7 +3770,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">Nº da peça 1 · 14:30–15:30 · motivo 10 (troca de inserto)
 </t>
@@ -3766,7 +3780,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">Certo: </t>
           </r>
@@ -3774,7 +3788,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">3 h de produção + 1 h parada = 4 h.
 </t>
@@ -3784,7 +3798,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">Errado: </t>
           </r>
@@ -3792,7 +3806,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="8.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>um trecho 13:00–17:00 com a parada dentro dele (a hora parada conta duas vezes).</t>
           </r>

</xml_diff>

<commit_message>
Excel: letras dos quadros de baixo ajustadas para a impressão do Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019Px7p5mhzWYWbE6aV5W89g
</commit_message>
<xml_diff>
--- a/docs/folha-modelo/diario-de-bordo.xlsx
+++ b/docs/folha-modelo/diario-de-bordo.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -143,11 +143,18 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="9.5"/>
+      <sz val="10.5"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10.5"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -350,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -463,6 +470,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1707,7 +1717,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">1. </t>
           </r>
@@ -1716,7 +1726,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Uma linha = uma peça.</t>
           </r>
@@ -1724,7 +1734,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> Começou peça nova? Linha nova.
 </t>
@@ -1733,7 +1743,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">2. </t>
           </r>
@@ -1742,7 +1752,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Trecho</t>
           </r>
@@ -1750,7 +1760,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> = tempo produzindo, </t>
           </r>
@@ -1759,7 +1769,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>sem parada no meio</t>
           </r>
@@ -1767,7 +1777,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">. Parou a máquina? </t>
           </r>
@@ -1776,7 +1786,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Feche o trecho</t>
           </r>
@@ -1784,7 +1794,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> (FIM).
 </t>
@@ -1793,7 +1803,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">3. Anote a parada no </t>
           </r>
@@ -1802,7 +1812,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>quadro 2</t>
           </r>
@@ -1810,7 +1820,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">, com o </t>
           </r>
@@ -1819,7 +1829,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Nº da peça</t>
           </r>
@@ -1827,7 +1837,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> e o código do motivo.
 </t>
@@ -1836,7 +1846,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">4. Voltou a produzir a mesma peça? Use o </t>
           </r>
@@ -1845,7 +1855,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>próximo trecho da mesma linha</t>
           </r>
@@ -1853,7 +1863,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">.
 </t>
@@ -1862,7 +1872,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">5. Troca de turno no meio da peça: o próximo operador usa o próximo trecho, com a chapa dele.
 </t>
@@ -1871,7 +1881,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">6. </t>
           </r>
@@ -1880,7 +1890,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Peça pronta?</t>
           </r>
@@ -1888,7 +1898,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> Escreva em </t>
           </r>
@@ -1897,7 +1907,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>PRONTA</t>
           </r>
@@ -1905,7 +1915,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> o </t>
           </r>
@@ -1914,7 +1924,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>turno que finalizou</t>
           </r>
@@ -1922,7 +1932,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> (1, 2 ou 3). Não terminou? Deixe em branco e continue na próxima folha.
 </t>
@@ -1931,7 +1941,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">7. </t>
           </r>
@@ -1940,7 +1950,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Mais de 4 trechos na mesma peça?</t>
           </r>
@@ -1948,7 +1958,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> Continue na </t>
           </r>
@@ -1957,7 +1967,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>linha de baixo</t>
           </r>
@@ -1965,7 +1975,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">, com a mesma peça, e escreva em </t>
           </r>
@@ -1974,7 +1984,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>CONTINUA A PEÇA Nº</t>
           </r>
@@ -1982,7 +1992,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> o número da linha de cima. O turno em PRONTA vai só na última linha.</t>
           </r>
@@ -1994,14 +2004,14 @@
       <c r="E32" s="35" t="n"/>
       <c r="F32" s="35" t="n"/>
       <c r="G32" s="36" t="n"/>
-      <c r="H32" s="18" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
+      <c r="H32" s="46" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="12"/>
             </rPr>
             <t>1</t>
           </r>
@@ -2009,7 +2019,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Mecânica
 </t>
@@ -2019,7 +2029,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>2</t>
           </r>
@@ -2027,7 +2037,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Elétrica
 </t>
@@ -2037,7 +2047,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>3</t>
           </r>
@@ -2045,7 +2055,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Manutenção preventiva
 </t>
@@ -2055,7 +2065,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>4</t>
           </r>
@@ -2063,7 +2073,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Troca de peça</t>
           </r>
@@ -2071,14 +2081,14 @@
       </c>
       <c r="I32" s="35" t="n"/>
       <c r="J32" s="36" t="n"/>
-      <c r="K32" s="18" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
+      <c r="K32" s="46" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="12"/>
             </rPr>
             <t>5</t>
           </r>
@@ -2086,7 +2096,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Falta de peça
 </t>
@@ -2096,7 +2106,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>6</t>
           </r>
@@ -2104,7 +2114,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Refeição
 </t>
@@ -2114,7 +2124,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>7</t>
           </r>
@@ -2122,7 +2132,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Tyorei
 </t>
@@ -2132,37 +2142,37 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
+              <sz val="12"/>
+            </rPr>
+            <t>8</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">  Outros (descreva)</t>
+          </r>
+        </is>
+      </c>
+      <c r="L32" s="36" t="n"/>
+      <c r="M32" s="47" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
               <sz val="11"/>
             </rPr>
-            <t>8</t>
+            <t xml:space="preserve">Quadro 1 (peça 1): </t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
               <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">  Outros (descreva)</t>
-          </r>
-        </is>
-      </c>
-      <c r="L32" s="36" t="n"/>
-      <c r="M32" s="46" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">Quadro 1 (peça 1): </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">VIGA · D51 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · Pronta: 1
 </t>
@@ -2172,7 +2182,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Quadro 2: </t>
           </r>
@@ -2180,7 +2190,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Nº da peça 1 · 14:30–15:30 · motivo 5 (falta de peça)
 </t>
@@ -2190,7 +2200,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Certo: </t>
           </r>
@@ -2198,7 +2208,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">3 h de produção + 1 h parada = 4 h.
 </t>
@@ -2208,7 +2218,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Errado: </t>
           </r>
@@ -2216,7 +2226,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t>um trecho 13:00–17:00 com a parada dentro dele (a hora parada conta duas vezes).</t>
           </r>
@@ -3261,7 +3271,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">1. </t>
           </r>
@@ -3270,7 +3280,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Uma linha = uma peça.</t>
           </r>
@@ -3278,7 +3288,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> Começou peça nova? Linha nova.
 </t>
@@ -3287,7 +3297,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">2. </t>
           </r>
@@ -3296,7 +3306,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Trecho</t>
           </r>
@@ -3304,7 +3314,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> = tempo produzindo, </t>
           </r>
@@ -3313,7 +3323,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>sem parada no meio</t>
           </r>
@@ -3321,7 +3331,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">. Parou a máquina? </t>
           </r>
@@ -3330,7 +3340,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Feche o trecho</t>
           </r>
@@ -3338,7 +3348,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> (FIM).
 </t>
@@ -3347,7 +3357,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">3. Anote a parada no </t>
           </r>
@@ -3356,7 +3366,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>quadro 2</t>
           </r>
@@ -3364,7 +3374,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">, com o </t>
           </r>
@@ -3373,7 +3383,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Nº da peça</t>
           </r>
@@ -3381,7 +3391,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> e o código do motivo.
 </t>
@@ -3390,7 +3400,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">4. Voltou a produzir a mesma peça? Use o </t>
           </r>
@@ -3399,7 +3409,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>próximo trecho da mesma linha</t>
           </r>
@@ -3407,7 +3417,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">.
 </t>
@@ -3416,7 +3426,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">5. Troca de turno no meio da peça: o próximo operador usa o próximo trecho, com a chapa dele.
 </t>
@@ -3425,7 +3435,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">6. </t>
           </r>
@@ -3434,7 +3444,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Peça pronta?</t>
           </r>
@@ -3442,7 +3452,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> Escreva em </t>
           </r>
@@ -3451,7 +3461,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>PRONTA</t>
           </r>
@@ -3459,7 +3469,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> o </t>
           </r>
@@ -3468,7 +3478,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>turno que finalizou</t>
           </r>
@@ -3476,7 +3486,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> (1, 2 ou 3). Não terminou? Deixe em branco e continue na próxima folha.
 </t>
@@ -3485,7 +3495,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">7. </t>
           </r>
@@ -3494,7 +3504,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>Mais de 4 trechos na mesma peça?</t>
           </r>
@@ -3502,7 +3512,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> Continue na </t>
           </r>
@@ -3511,7 +3521,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>linha de baixo</t>
           </r>
@@ -3519,7 +3529,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">, com a mesma peça, e escreva em </t>
           </r>
@@ -3528,7 +3538,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t>CONTINUA A PEÇA Nº</t>
           </r>
@@ -3536,7 +3546,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="9.5"/>
+              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve"> o número da linha de cima. O turno em PRONTA vai só na última linha.</t>
           </r>
@@ -3548,14 +3558,14 @@
       <c r="E32" s="35" t="n"/>
       <c r="F32" s="35" t="n"/>
       <c r="G32" s="36" t="n"/>
-      <c r="H32" s="18" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
+      <c r="H32" s="46" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="12"/>
             </rPr>
             <t>1</t>
           </r>
@@ -3563,7 +3573,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Mecânica
 </t>
@@ -3573,7 +3583,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>2</t>
           </r>
@@ -3581,7 +3591,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Elétrica
 </t>
@@ -3591,7 +3601,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>3</t>
           </r>
@@ -3599,7 +3609,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Manutenção preventiva
 </t>
@@ -3609,7 +3619,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>4</t>
           </r>
@@ -3617,7 +3627,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Troca de peça
 </t>
@@ -3627,7 +3637,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>5</t>
           </r>
@@ -3635,7 +3645,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Falta de peça</t>
           </r>
@@ -3643,14 +3653,14 @@
       </c>
       <c r="I32" s="35" t="n"/>
       <c r="J32" s="36" t="n"/>
-      <c r="K32" s="18" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
+      <c r="K32" s="46" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="12"/>
             </rPr>
             <t>6</t>
           </r>
@@ -3658,7 +3668,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Refeição
 </t>
@@ -3668,7 +3678,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>7</t>
           </r>
@@ -3676,7 +3686,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Tyorei
 </t>
@@ -3686,7 +3696,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>8</t>
           </r>
@@ -3694,7 +3704,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Outros (descreva)
 </t>
@@ -3704,7 +3714,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t>9</t>
           </r>
@@ -3712,7 +3722,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="11"/>
+              <sz val="12"/>
             </rPr>
             <t xml:space="preserve">  Set-up
 </t>
@@ -3722,37 +3732,37 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
+              <sz val="12"/>
+            </rPr>
+            <t>10</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">  Ferramenta</t>
+          </r>
+        </is>
+      </c>
+      <c r="L32" s="36" t="n"/>
+      <c r="M32" s="47" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
               <sz val="11"/>
             </rPr>
-            <t>10</t>
+            <t xml:space="preserve">Quadro 1 (peça 1): </t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
               <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">  Ferramenta</t>
-          </r>
-        </is>
-      </c>
-      <c r="L32" s="36" t="n"/>
-      <c r="M32" s="46" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">Quadro 1 (peça 1): </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">MESA · D61 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · Pronta: 1
 </t>
@@ -3762,7 +3772,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Quadro 2: </t>
           </r>
@@ -3770,7 +3780,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Nº da peça 1 · 14:30–15:30 · motivo 10 (troca de inserto)
 </t>
@@ -3780,7 +3790,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Certo: </t>
           </r>
@@ -3788,7 +3798,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">3 h de produção + 1 h parada = 4 h.
 </t>
@@ -3798,7 +3808,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t xml:space="preserve">Errado: </t>
           </r>
@@ -3806,7 +3816,7 @@
             <rPr>
               <rFont val="Arial"/>
               <color rgb="FF111111"/>
-              <sz val="10.5"/>
+              <sz val="11"/>
             </rPr>
             <t>um trecho 13:00–17:00 com a parada dentro dele (a hora parada conta duas vezes).</t>
           </r>

</xml_diff>

<commit_message>
Folhas A4: 12 linhas de produção e quadros de baixo com uma frase por linha (sem quebra, reduz para caber)
Assim a impressão sai igual no Excel e no PDF.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019Px7p5mhzWYWbE6aV5W89g
</commit_message>
<xml_diff>
--- a/docs/folha-modelo/diario-de-bordo.xlsx
+++ b/docs/folha-modelo/diario-de-bordo.xlsx
@@ -11,8 +11,8 @@
     <sheet name="A3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'A4 Robô'!$A$1:$S$38</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'A4 Usinagem'!$A$1:$S$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'A4 Robô'!$A$1:$S$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'A4 Usinagem'!$A$1:$S$40</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'A3'!$A$1:$S$64</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -156,6 +156,10 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -185,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -353,11 +357,70 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+    </border>
+    <border/>
+    <border>
+      <right style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <top style="thin"/>
+    </border>
+    <border>
+      <top style="thin"/>
+    </border>
+    <border>
+      <right style="thin"/>
+      <top style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <right style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -478,6 +541,26 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -843,7 +926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S38"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.05" customWidth="1" min="1" max="1"/>
@@ -1363,102 +1446,69 @@
       <c r="R16" s="13" t="n"/>
       <c r="S16" s="16" t="n"/>
     </row>
-    <row r="17" ht="17.1" customHeight="1">
-      <c r="A17" s="26" t="inlineStr">
+    <row r="17" ht="21" customHeight="1">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="11" t="n"/>
+      <c r="J17" s="11" t="n"/>
+      <c r="K17" s="7" t="n"/>
+      <c r="L17" s="11" t="n"/>
+      <c r="M17" s="11" t="n"/>
+      <c r="N17" s="7" t="n"/>
+      <c r="O17" s="11" t="n"/>
+      <c r="P17" s="11" t="n"/>
+      <c r="Q17" s="9" t="n"/>
+      <c r="R17" s="13" t="n"/>
+      <c r="S17" s="16" t="n"/>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="11" t="n"/>
+      <c r="J18" s="11" t="n"/>
+      <c r="K18" s="7" t="n"/>
+      <c r="L18" s="11" t="n"/>
+      <c r="M18" s="11" t="n"/>
+      <c r="N18" s="7" t="n"/>
+      <c r="O18" s="11" t="n"/>
+      <c r="P18" s="11" t="n"/>
+      <c r="Q18" s="9" t="n"/>
+      <c r="R18" s="13" t="n"/>
+      <c r="S18" s="16" t="n"/>
+    </row>
+    <row r="19" ht="17.1" customHeight="1">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>2. PARADAS DA MÁQUINA</t>
         </is>
       </c>
-      <c r="B17" s="38" t="n"/>
-      <c r="C17" s="38" t="n"/>
-      <c r="D17" s="38" t="n"/>
-      <c r="E17" s="38" t="n"/>
-      <c r="F17" s="38" t="n"/>
-      <c r="G17" s="38" t="n"/>
-      <c r="H17" s="37" t="n"/>
-      <c r="I17" s="22" t="inlineStr">
+      <c r="B19" s="38" t="n"/>
+      <c r="C19" s="38" t="n"/>
+      <c r="D19" s="38" t="n"/>
+      <c r="E19" s="38" t="n"/>
+      <c r="F19" s="38" t="n"/>
+      <c r="G19" s="38" t="n"/>
+      <c r="H19" s="37" t="n"/>
+      <c r="I19" s="22" t="inlineStr">
         <is>
           <t>escreva o Nº da peça que estava na máquina (ou “—” se não havia peça)</t>
         </is>
       </c>
-      <c r="J17" s="38" t="n"/>
-      <c r="K17" s="38" t="n"/>
-      <c r="L17" s="38" t="n"/>
-      <c r="M17" s="38" t="n"/>
-      <c r="N17" s="38" t="n"/>
-      <c r="O17" s="38" t="n"/>
-      <c r="P17" s="38" t="n"/>
-      <c r="Q17" s="38" t="n"/>
-      <c r="R17" s="38" t="n"/>
-      <c r="S17" s="37" t="n"/>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Nº</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>TURNO</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="inlineStr">
-        <is>
-          <t>DATA</t>
-        </is>
-      </c>
-      <c r="D18" s="17" t="inlineStr">
-        <is>
-          <t>CHAPA</t>
-        </is>
-      </c>
-      <c r="E18" s="17" t="inlineStr">
-        <is>
-          <t>INÍCIO</t>
-        </is>
-      </c>
-      <c r="F18" s="37" t="n"/>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>FIM</t>
-        </is>
-      </c>
-      <c r="H18" s="37" t="n"/>
-      <c r="I18" s="17" t="inlineStr">
-        <is>
-          <t>MOTIVO
-(código 1–8)</t>
-        </is>
-      </c>
-      <c r="J18" s="38" t="n"/>
-      <c r="K18" s="37" t="n"/>
-      <c r="L18" s="17" t="inlineStr">
-        <is>
-          <t>DESCRIÇÃO DA PARADA</t>
-        </is>
-      </c>
-      <c r="M18" s="38" t="n"/>
-      <c r="N18" s="38" t="n"/>
-      <c r="O18" s="38" t="n"/>
-      <c r="P18" s="38" t="n"/>
-      <c r="Q18" s="38" t="n"/>
-      <c r="R18" s="38" t="n"/>
-      <c r="S18" s="37" t="n"/>
-    </row>
-    <row r="19" ht="18.95" customHeight="1">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="13" t="n"/>
-      <c r="C19" s="13" t="n"/>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="37" t="n"/>
-      <c r="G19" s="11" t="n"/>
-      <c r="H19" s="37" t="n"/>
-      <c r="I19" s="31" t="n"/>
-      <c r="J19" s="34" t="n"/>
-      <c r="K19" s="32" t="n"/>
-      <c r="L19" s="16" t="n"/>
+      <c r="J19" s="38" t="n"/>
+      <c r="K19" s="38" t="n"/>
+      <c r="L19" s="38" t="n"/>
       <c r="M19" s="38" t="n"/>
       <c r="N19" s="38" t="n"/>
       <c r="O19" s="38" t="n"/>
@@ -1467,19 +1517,52 @@
       <c r="R19" s="38" t="n"/>
       <c r="S19" s="37" t="n"/>
     </row>
-    <row r="20" ht="18.95" customHeight="1">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="11" t="n"/>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>TURNO</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>CHAPA</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>INÍCIO</t>
+        </is>
+      </c>
       <c r="F20" s="37" t="n"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>FIM</t>
+        </is>
+      </c>
       <c r="H20" s="37" t="n"/>
-      <c r="I20" s="31" t="n"/>
-      <c r="J20" s="34" t="n"/>
-      <c r="K20" s="32" t="n"/>
-      <c r="L20" s="16" t="n"/>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>MOTIVO
+(código 1–8)</t>
+        </is>
+      </c>
+      <c r="J20" s="38" t="n"/>
+      <c r="K20" s="37" t="n"/>
+      <c r="L20" s="17" t="inlineStr">
+        <is>
+          <t>DESCRIÇÃO DA PARADA</t>
+        </is>
+      </c>
       <c r="M20" s="38" t="n"/>
       <c r="N20" s="38" t="n"/>
       <c r="O20" s="38" t="n"/>
@@ -1677,32 +1760,41 @@
       <c r="R29" s="38" t="n"/>
       <c r="S29" s="37" t="n"/>
     </row>
-    <row r="31">
-      <c r="A31" s="21" t="inlineStr">
-        <is>
-          <t>COMO PREENCHER</t>
-        </is>
-      </c>
-      <c r="B31" s="38" t="n"/>
-      <c r="C31" s="38" t="n"/>
-      <c r="D31" s="38" t="n"/>
-      <c r="E31" s="38" t="n"/>
-      <c r="F31" s="38" t="n"/>
-      <c r="G31" s="37" t="n"/>
-      <c r="H31" s="21" t="inlineStr">
-        <is>
-          <t>CÓDIGOS DE PARADA (coluna MOTIVO)</t>
-        </is>
-      </c>
-      <c r="I31" s="38" t="n"/>
-      <c r="J31" s="38" t="n"/>
-      <c r="K31" s="38" t="n"/>
-      <c r="L31" s="37" t="n"/>
-      <c r="M31" s="21" t="inlineStr">
-        <is>
-          <t>EXEMPLO: VIGA D51, 13:00 ÀS 17:00, PAROU 14:30–15:30</t>
-        </is>
-      </c>
+    <row r="30" ht="18.95" customHeight="1">
+      <c r="A30" s="6" t="n"/>
+      <c r="B30" s="13" t="n"/>
+      <c r="C30" s="13" t="n"/>
+      <c r="D30" s="13" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="37" t="n"/>
+      <c r="G30" s="11" t="n"/>
+      <c r="H30" s="37" t="n"/>
+      <c r="I30" s="31" t="n"/>
+      <c r="J30" s="34" t="n"/>
+      <c r="K30" s="32" t="n"/>
+      <c r="L30" s="16" t="n"/>
+      <c r="M30" s="38" t="n"/>
+      <c r="N30" s="38" t="n"/>
+      <c r="O30" s="38" t="n"/>
+      <c r="P30" s="38" t="n"/>
+      <c r="Q30" s="38" t="n"/>
+      <c r="R30" s="38" t="n"/>
+      <c r="S30" s="37" t="n"/>
+    </row>
+    <row r="31" ht="18.95" customHeight="1">
+      <c r="A31" s="6" t="n"/>
+      <c r="B31" s="13" t="n"/>
+      <c r="C31" s="13" t="n"/>
+      <c r="D31" s="13" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="37" t="n"/>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="37" t="n"/>
+      <c r="I31" s="31" t="n"/>
+      <c r="J31" s="34" t="n"/>
+      <c r="K31" s="32" t="n"/>
+      <c r="L31" s="16" t="n"/>
+      <c r="M31" s="38" t="n"/>
       <c r="N31" s="38" t="n"/>
       <c r="O31" s="38" t="n"/>
       <c r="P31" s="38" t="n"/>
@@ -1710,679 +1802,606 @@
       <c r="R31" s="38" t="n"/>
       <c r="S31" s="37" t="n"/>
     </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="45" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">1. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Uma linha = uma peça.</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> Começou peça nova? Linha nova.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">2. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Trecho</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> = tempo produzindo, </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>sem parada no meio</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">. Parou a máquina? </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Feche o trecho</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> (FIM).
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">3. Anote a parada no </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>quadro 2</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">, com o </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Nº da peça</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> e o código do motivo.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">4. Voltou a produzir a mesma peça? Use o </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>próximo trecho da mesma linha</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">5. Troca de turno no meio da peça: o próximo operador usa o próximo trecho, com a chapa dele.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">6. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Peça pronta?</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> Escreva em </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>PRONTA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> o </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>turno que finalizou</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> (1, 2 ou 3). Não terminou? Deixe em branco e continue na próxima folha.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">7. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Mais de 4 trechos na mesma peça?</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> Continue na </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>linha de baixo</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">, com a mesma peça, e escreva em </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>CONTINUA A PEÇA Nº</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> o número da linha de cima. O turno em PRONTA vai só na última linha.</t>
-          </r>
-        </is>
-      </c>
-      <c r="B32" s="35" t="n"/>
-      <c r="C32" s="35" t="n"/>
-      <c r="D32" s="35" t="n"/>
-      <c r="E32" s="35" t="n"/>
-      <c r="F32" s="35" t="n"/>
-      <c r="G32" s="36" t="n"/>
-      <c r="H32" s="46" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+    <row r="32" ht="6" customHeight="1"/>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>COMO PREENCHER</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="n"/>
+      <c r="C33" s="38" t="n"/>
+      <c r="D33" s="38" t="n"/>
+      <c r="E33" s="38" t="n"/>
+      <c r="F33" s="38" t="n"/>
+      <c r="G33" s="37" t="n"/>
+      <c r="H33" s="21" t="inlineStr">
+        <is>
+          <t>CÓDIGOS DE PARADA (coluna MOTIVO)</t>
+        </is>
+      </c>
+      <c r="I33" s="38" t="n"/>
+      <c r="J33" s="38" t="n"/>
+      <c r="K33" s="38" t="n"/>
+      <c r="L33" s="37" t="n"/>
+      <c r="M33" s="21" t="inlineStr">
+        <is>
+          <t>EXEMPLO: VIGA D51, 13:00 ÀS 17:00, PAROU 14:30–15:30</t>
+        </is>
+      </c>
+      <c r="N33" s="38" t="n"/>
+      <c r="O33" s="38" t="n"/>
+      <c r="P33" s="38" t="n"/>
+      <c r="Q33" s="38" t="n"/>
+      <c r="R33" s="38" t="n"/>
+      <c r="S33" s="37" t="n"/>
+    </row>
+    <row r="34" ht="13.5" customHeight="1">
+      <c r="A34" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>1. Uma linha = uma peça.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Começou peça nova? Linha nova.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G34" s="49" t="n"/>
+      <c r="H34" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
             </rPr>
             <t>1</t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Mecânica
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Mecânica</t>
+          </r>
+        </is>
+      </c>
+      <c r="J34" s="49" t="n"/>
+      <c r="K34" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>5</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Falta de peça</t>
+          </r>
+        </is>
+      </c>
+      <c r="L34" s="49" t="n"/>
+      <c r="M34" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Quadro 1 (peça 1):</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> VIGA · D51 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · Pronta: 1</t>
+          </r>
+        </is>
+      </c>
+      <c r="S34" s="49" t="n"/>
+    </row>
+    <row r="35" ht="13.5" customHeight="1">
+      <c r="A35" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>2. Trecho = só produção.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Parou a máquina? Escreva o FIM do trecho.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
             </rPr>
             <t>2</t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Elétrica
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Elétrica</t>
+          </r>
+        </is>
+      </c>
+      <c r="J35" s="49" t="n"/>
+      <c r="K35" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>6</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Refeição</t>
+          </r>
+        </is>
+      </c>
+      <c r="L35" s="49" t="n"/>
+      <c r="M35" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Quadro 2:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Nº da peça 1 · 14:30–15:30 · motivo 5 (falta de peça)</t>
+          </r>
+        </is>
+      </c>
+      <c r="S35" s="49" t="n"/>
+    </row>
+    <row r="36" ht="13.5" customHeight="1">
+      <c r="A36" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>3. Anote a parada no quadro 2,</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> com o Nº da peça e o código do motivo.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
             </rPr>
             <t>3</t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Manutenção preventiva
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Manutenção preventiva</t>
+          </r>
+        </is>
+      </c>
+      <c r="J36" s="49" t="n"/>
+      <c r="K36" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>7</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Tyorei</t>
+          </r>
+        </is>
+      </c>
+      <c r="L36" s="49" t="n"/>
+      <c r="M36" s="48" t="n"/>
+      <c r="S36" s="49" t="n"/>
+    </row>
+    <row r="37" ht="13.5" customHeight="1">
+      <c r="A37" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>4. Voltou a produzir a mesma peça?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Use o próximo trecho da mesma linha.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G37" s="49" t="n"/>
+      <c r="H37" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
             </rPr>
             <t>4</t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+              <sz val="9"/>
             </rPr>
             <t xml:space="preserve">  Troca de peça</t>
           </r>
         </is>
       </c>
-      <c r="I32" s="35" t="n"/>
-      <c r="J32" s="36" t="n"/>
-      <c r="K32" s="46" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t>5</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Falta de peça
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t>6</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Refeição
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t>7</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Tyorei
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+      <c r="J37" s="49" t="n"/>
+      <c r="K37" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
             </rPr>
             <t>8</t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+              <sz val="9"/>
             </rPr>
             <t xml:space="preserve">  Outros (descreva)</t>
           </r>
         </is>
       </c>
-      <c r="L32" s="36" t="n"/>
-      <c r="M32" s="47" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Quadro 1 (peça 1): </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">VIGA · D51 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · Pronta: 1
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Quadro 2: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Nº da peça 1 · 14:30–15:30 · motivo 5 (falta de peça)
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Certo: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">3 h de produção + 1 h parada = 4 h.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Errado: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t>um trecho 13:00–17:00 com a parada dentro dele (a hora parada conta duas vezes).</t>
-          </r>
-        </is>
-      </c>
-      <c r="N32" s="35" t="n"/>
-      <c r="O32" s="35" t="n"/>
-      <c r="P32" s="35" t="n"/>
-      <c r="Q32" s="35" t="n"/>
-      <c r="R32" s="35" t="n"/>
-      <c r="S32" s="36" t="n"/>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="43" t="n"/>
-      <c r="G33" s="44" t="n"/>
-      <c r="H33" s="43" t="n"/>
-      <c r="J33" s="44" t="n"/>
-      <c r="K33" s="43" t="n"/>
-      <c r="L33" s="44" t="n"/>
-      <c r="M33" s="43" t="n"/>
-      <c r="S33" s="44" t="n"/>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="43" t="n"/>
-      <c r="G34" s="44" t="n"/>
-      <c r="H34" s="43" t="n"/>
-      <c r="J34" s="44" t="n"/>
-      <c r="K34" s="43" t="n"/>
-      <c r="L34" s="44" t="n"/>
-      <c r="M34" s="43" t="n"/>
-      <c r="S34" s="44" t="n"/>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="43" t="n"/>
-      <c r="G35" s="44" t="n"/>
-      <c r="H35" s="43" t="n"/>
-      <c r="J35" s="44" t="n"/>
-      <c r="K35" s="43" t="n"/>
-      <c r="L35" s="44" t="n"/>
-      <c r="M35" s="43" t="n"/>
-      <c r="S35" s="44" t="n"/>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="43" t="n"/>
-      <c r="G36" s="44" t="n"/>
-      <c r="H36" s="43" t="n"/>
-      <c r="J36" s="44" t="n"/>
-      <c r="K36" s="43" t="n"/>
-      <c r="L36" s="44" t="n"/>
-      <c r="M36" s="43" t="n"/>
-      <c r="S36" s="44" t="n"/>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="43" t="n"/>
-      <c r="G37" s="44" t="n"/>
-      <c r="H37" s="43" t="n"/>
-      <c r="J37" s="44" t="n"/>
-      <c r="K37" s="43" t="n"/>
-      <c r="L37" s="44" t="n"/>
-      <c r="M37" s="43" t="n"/>
-      <c r="S37" s="44" t="n"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="39" t="n"/>
-      <c r="B38" s="40" t="n"/>
-      <c r="C38" s="40" t="n"/>
-      <c r="D38" s="40" t="n"/>
-      <c r="E38" s="40" t="n"/>
-      <c r="F38" s="40" t="n"/>
-      <c r="G38" s="41" t="n"/>
-      <c r="H38" s="39" t="n"/>
-      <c r="I38" s="40" t="n"/>
-      <c r="J38" s="41" t="n"/>
-      <c r="K38" s="39" t="n"/>
-      <c r="L38" s="41" t="n"/>
-      <c r="M38" s="39" t="n"/>
-      <c r="N38" s="40" t="n"/>
-      <c r="O38" s="40" t="n"/>
-      <c r="P38" s="40" t="n"/>
-      <c r="Q38" s="40" t="n"/>
-      <c r="R38" s="40" t="n"/>
-      <c r="S38" s="41" t="n"/>
-    </row>
+      <c r="L37" s="49" t="n"/>
+      <c r="M37" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Certo:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> 3 h produzindo + 1 h parado = 4 h.</t>
+          </r>
+        </is>
+      </c>
+      <c r="S37" s="49" t="n"/>
+    </row>
+    <row r="38" ht="13.5" customHeight="1">
+      <c r="A38" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>5. Trocou o turno no meio da peça?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> O próximo operador usa o próximo trecho, com a chapa dele.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G38" s="49" t="n"/>
+      <c r="H38" s="50" t="n"/>
+      <c r="J38" s="49" t="n"/>
+      <c r="K38" s="50" t="n"/>
+      <c r="L38" s="49" t="n"/>
+      <c r="M38" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Errado:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> um trecho só, 13:00–17:00, com a parada dentro dele.</t>
+          </r>
+        </is>
+      </c>
+      <c r="S38" s="49" t="n"/>
+    </row>
+    <row r="39" ht="13.5" customHeight="1">
+      <c r="A39" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>6. Peça pronta?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Escreva em PRONTA o turno (1, 2 ou 3). Não terminou? Deixe em branco.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G39" s="49" t="n"/>
+      <c r="H39" s="51" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Sem peça na máquina?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> No Nº da parada, escreva —</t>
+          </r>
+        </is>
+      </c>
+      <c r="I39" s="52" t="n"/>
+      <c r="J39" s="52" t="n"/>
+      <c r="K39" s="52" t="n"/>
+      <c r="L39" s="53" t="n"/>
+      <c r="M39" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t>A hora parada contaria duas vezes.</t>
+          </r>
+        </is>
+      </c>
+      <c r="S39" s="49" t="n"/>
+    </row>
+    <row r="40" ht="13.5" customHeight="1">
+      <c r="A40" s="54" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>7. Mais de 4 trechos?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Siga na linha de baixo e escreva em CONTINUA o Nº da linha de cima.</t>
+          </r>
+        </is>
+      </c>
+      <c r="B40" s="55" t="n"/>
+      <c r="C40" s="55" t="n"/>
+      <c r="D40" s="55" t="n"/>
+      <c r="E40" s="55" t="n"/>
+      <c r="F40" s="55" t="n"/>
+      <c r="G40" s="56" t="n"/>
+      <c r="H40" s="57" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Parada fora da lista?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Use o código 8 e descreva.</t>
+          </r>
+        </is>
+      </c>
+      <c r="I40" s="58" t="n"/>
+      <c r="J40" s="58" t="n"/>
+      <c r="K40" s="58" t="n"/>
+      <c r="L40" s="59" t="n"/>
+      <c r="M40" s="54" t="n"/>
+      <c r="N40" s="55" t="n"/>
+      <c r="O40" s="55" t="n"/>
+      <c r="P40" s="55" t="n"/>
+      <c r="Q40" s="55" t="n"/>
+      <c r="R40" s="55" t="n"/>
+      <c r="S40" s="56" t="n"/>
+    </row>
+    <row r="41"/>
   </sheetData>
-  <mergeCells count="72">
+  <mergeCells count="94">
+    <mergeCell ref="M36:S36"/>
     <mergeCell ref="G21:H21"/>
+    <mergeCell ref="M33:S33"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="M38:S38"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="L24:S24"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="L30:S30"/>
+    <mergeCell ref="L26:S26"/>
+    <mergeCell ref="L20:S20"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="L29:S29"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="L22:S22"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="L31:S31"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="R5:R6"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="L21:S21"/>
+    <mergeCell ref="H33:L33"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="L27:S27"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="K37:L37"/>
     <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="H36:J36"/>
     <mergeCell ref="E24:F24"/>
     <mergeCell ref="G27:H27"/>
     <mergeCell ref="N5:P5"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="L19:S19"/>
-    <mergeCell ref="G23:H23"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="L28:S28"/>
-    <mergeCell ref="H31:L31"/>
-    <mergeCell ref="A32:G38"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="M32:S38"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="A1:L2"/>
-    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="H40:L40"/>
+    <mergeCell ref="H39:L39"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="H37:J37"/>
     <mergeCell ref="E28:F28"/>
-    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="M37:S37"/>
     <mergeCell ref="G28:H28"/>
-    <mergeCell ref="L24:S24"/>
-    <mergeCell ref="L18:S18"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="K32:L38"/>
-    <mergeCell ref="L23:S23"/>
+    <mergeCell ref="M34:S34"/>
+    <mergeCell ref="Q2:S2"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="A5:A6"/>
-    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="L23:S23"/>
+    <mergeCell ref="A36:G36"/>
     <mergeCell ref="S5:S6"/>
-    <mergeCell ref="H32:J38"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="M39:S39"/>
+    <mergeCell ref="G30:H30"/>
     <mergeCell ref="G24:H24"/>
-    <mergeCell ref="L20:S20"/>
-    <mergeCell ref="L26:S26"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="L29:S29"/>
-    <mergeCell ref="E27:F27"/>
     <mergeCell ref="L25:S25"/>
-    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="M35:S35"/>
+    <mergeCell ref="H35:J35"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="L22:S22"/>
     <mergeCell ref="G26:H26"/>
     <mergeCell ref="D5:D6"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="A4:H4"/>
     <mergeCell ref="G29:H29"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="R5:R6"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="I17:S17"/>
-    <mergeCell ref="M31:S31"/>
     <mergeCell ref="I4:S4"/>
     <mergeCell ref="E5:G5"/>
     <mergeCell ref="E25:F25"/>
-    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="K38:L38"/>
     <mergeCell ref="G25:H25"/>
-    <mergeCell ref="L21:S21"/>
+    <mergeCell ref="M40:S40"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="I19:S19"/>
+    <mergeCell ref="A33:G33"/>
     <mergeCell ref="E21:F21"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="L27:S27"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="K3:L3"/>
     <mergeCell ref="C5:C6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
@@ -2397,7 +2416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S38"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.05" customWidth="1" min="1" max="1"/>
@@ -2917,102 +2936,69 @@
       <c r="R16" s="13" t="n"/>
       <c r="S16" s="16" t="n"/>
     </row>
-    <row r="17" ht="17.1" customHeight="1">
-      <c r="A17" s="26" t="inlineStr">
+    <row r="17" ht="21" customHeight="1">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="11" t="n"/>
+      <c r="J17" s="11" t="n"/>
+      <c r="K17" s="7" t="n"/>
+      <c r="L17" s="11" t="n"/>
+      <c r="M17" s="11" t="n"/>
+      <c r="N17" s="7" t="n"/>
+      <c r="O17" s="11" t="n"/>
+      <c r="P17" s="11" t="n"/>
+      <c r="Q17" s="9" t="n"/>
+      <c r="R17" s="13" t="n"/>
+      <c r="S17" s="16" t="n"/>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="11" t="n"/>
+      <c r="J18" s="11" t="n"/>
+      <c r="K18" s="7" t="n"/>
+      <c r="L18" s="11" t="n"/>
+      <c r="M18" s="11" t="n"/>
+      <c r="N18" s="7" t="n"/>
+      <c r="O18" s="11" t="n"/>
+      <c r="P18" s="11" t="n"/>
+      <c r="Q18" s="9" t="n"/>
+      <c r="R18" s="13" t="n"/>
+      <c r="S18" s="16" t="n"/>
+    </row>
+    <row r="19" ht="17.1" customHeight="1">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>2. PARADAS DA MÁQUINA</t>
         </is>
       </c>
-      <c r="B17" s="38" t="n"/>
-      <c r="C17" s="38" t="n"/>
-      <c r="D17" s="38" t="n"/>
-      <c r="E17" s="38" t="n"/>
-      <c r="F17" s="38" t="n"/>
-      <c r="G17" s="38" t="n"/>
-      <c r="H17" s="37" t="n"/>
-      <c r="I17" s="22" t="inlineStr">
+      <c r="B19" s="38" t="n"/>
+      <c r="C19" s="38" t="n"/>
+      <c r="D19" s="38" t="n"/>
+      <c r="E19" s="38" t="n"/>
+      <c r="F19" s="38" t="n"/>
+      <c r="G19" s="38" t="n"/>
+      <c r="H19" s="37" t="n"/>
+      <c r="I19" s="22" t="inlineStr">
         <is>
           <t>escreva o Nº da peça que estava na máquina (ou “—” se não havia peça)</t>
         </is>
       </c>
-      <c r="J17" s="38" t="n"/>
-      <c r="K17" s="38" t="n"/>
-      <c r="L17" s="38" t="n"/>
-      <c r="M17" s="38" t="n"/>
-      <c r="N17" s="38" t="n"/>
-      <c r="O17" s="38" t="n"/>
-      <c r="P17" s="38" t="n"/>
-      <c r="Q17" s="38" t="n"/>
-      <c r="R17" s="38" t="n"/>
-      <c r="S17" s="37" t="n"/>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Nº</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>TURNO</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="inlineStr">
-        <is>
-          <t>DATA</t>
-        </is>
-      </c>
-      <c r="D18" s="17" t="inlineStr">
-        <is>
-          <t>CHAPA</t>
-        </is>
-      </c>
-      <c r="E18" s="17" t="inlineStr">
-        <is>
-          <t>INÍCIO</t>
-        </is>
-      </c>
-      <c r="F18" s="37" t="n"/>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>FIM</t>
-        </is>
-      </c>
-      <c r="H18" s="37" t="n"/>
-      <c r="I18" s="17" t="inlineStr">
-        <is>
-          <t>MOTIVO
-(código 1–10)</t>
-        </is>
-      </c>
-      <c r="J18" s="38" t="n"/>
-      <c r="K18" s="37" t="n"/>
-      <c r="L18" s="17" t="inlineStr">
-        <is>
-          <t>DESCRIÇÃO DA PARADA</t>
-        </is>
-      </c>
-      <c r="M18" s="38" t="n"/>
-      <c r="N18" s="38" t="n"/>
-      <c r="O18" s="38" t="n"/>
-      <c r="P18" s="38" t="n"/>
-      <c r="Q18" s="38" t="n"/>
-      <c r="R18" s="38" t="n"/>
-      <c r="S18" s="37" t="n"/>
-    </row>
-    <row r="19" ht="18.95" customHeight="1">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="13" t="n"/>
-      <c r="C19" s="13" t="n"/>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="37" t="n"/>
-      <c r="G19" s="11" t="n"/>
-      <c r="H19" s="37" t="n"/>
-      <c r="I19" s="31" t="n"/>
-      <c r="J19" s="34" t="n"/>
-      <c r="K19" s="32" t="n"/>
-      <c r="L19" s="16" t="n"/>
+      <c r="J19" s="38" t="n"/>
+      <c r="K19" s="38" t="n"/>
+      <c r="L19" s="38" t="n"/>
       <c r="M19" s="38" t="n"/>
       <c r="N19" s="38" t="n"/>
       <c r="O19" s="38" t="n"/>
@@ -3021,19 +3007,52 @@
       <c r="R19" s="38" t="n"/>
       <c r="S19" s="37" t="n"/>
     </row>
-    <row r="20" ht="18.95" customHeight="1">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="11" t="n"/>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>TURNO</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>CHAPA</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>INÍCIO</t>
+        </is>
+      </c>
       <c r="F20" s="37" t="n"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>FIM</t>
+        </is>
+      </c>
       <c r="H20" s="37" t="n"/>
-      <c r="I20" s="31" t="n"/>
-      <c r="J20" s="34" t="n"/>
-      <c r="K20" s="32" t="n"/>
-      <c r="L20" s="16" t="n"/>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>MOTIVO
+(código 1–10)</t>
+        </is>
+      </c>
+      <c r="J20" s="38" t="n"/>
+      <c r="K20" s="37" t="n"/>
+      <c r="L20" s="17" t="inlineStr">
+        <is>
+          <t>DESCRIÇÃO DA PARADA</t>
+        </is>
+      </c>
       <c r="M20" s="38" t="n"/>
       <c r="N20" s="38" t="n"/>
       <c r="O20" s="38" t="n"/>
@@ -3231,32 +3250,41 @@
       <c r="R29" s="38" t="n"/>
       <c r="S29" s="37" t="n"/>
     </row>
-    <row r="31">
-      <c r="A31" s="21" t="inlineStr">
-        <is>
-          <t>COMO PREENCHER</t>
-        </is>
-      </c>
-      <c r="B31" s="38" t="n"/>
-      <c r="C31" s="38" t="n"/>
-      <c r="D31" s="38" t="n"/>
-      <c r="E31" s="38" t="n"/>
-      <c r="F31" s="38" t="n"/>
-      <c r="G31" s="37" t="n"/>
-      <c r="H31" s="21" t="inlineStr">
-        <is>
-          <t>CÓDIGOS DE PARADA (coluna MOTIVO)</t>
-        </is>
-      </c>
-      <c r="I31" s="38" t="n"/>
-      <c r="J31" s="38" t="n"/>
-      <c r="K31" s="38" t="n"/>
-      <c r="L31" s="37" t="n"/>
-      <c r="M31" s="21" t="inlineStr">
-        <is>
-          <t>EXEMPLO: MESA D61, 13:00 ÀS 17:00, PAROU 14:30–15:30</t>
-        </is>
-      </c>
+    <row r="30" ht="18.95" customHeight="1">
+      <c r="A30" s="6" t="n"/>
+      <c r="B30" s="13" t="n"/>
+      <c r="C30" s="13" t="n"/>
+      <c r="D30" s="13" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="37" t="n"/>
+      <c r="G30" s="11" t="n"/>
+      <c r="H30" s="37" t="n"/>
+      <c r="I30" s="31" t="n"/>
+      <c r="J30" s="34" t="n"/>
+      <c r="K30" s="32" t="n"/>
+      <c r="L30" s="16" t="n"/>
+      <c r="M30" s="38" t="n"/>
+      <c r="N30" s="38" t="n"/>
+      <c r="O30" s="38" t="n"/>
+      <c r="P30" s="38" t="n"/>
+      <c r="Q30" s="38" t="n"/>
+      <c r="R30" s="38" t="n"/>
+      <c r="S30" s="37" t="n"/>
+    </row>
+    <row r="31" ht="18.95" customHeight="1">
+      <c r="A31" s="6" t="n"/>
+      <c r="B31" s="13" t="n"/>
+      <c r="C31" s="13" t="n"/>
+      <c r="D31" s="13" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="37" t="n"/>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="37" t="n"/>
+      <c r="I31" s="31" t="n"/>
+      <c r="J31" s="34" t="n"/>
+      <c r="K31" s="32" t="n"/>
+      <c r="L31" s="16" t="n"/>
+      <c r="M31" s="38" t="n"/>
       <c r="N31" s="38" t="n"/>
       <c r="O31" s="38" t="n"/>
       <c r="P31" s="38" t="n"/>
@@ -3264,715 +3292,642 @@
       <c r="R31" s="38" t="n"/>
       <c r="S31" s="37" t="n"/>
     </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="45" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">1. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Uma linha = uma peça.</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> Começou peça nova? Linha nova.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">2. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Trecho</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> = tempo produzindo, </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>sem parada no meio</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">. Parou a máquina? </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Feche o trecho</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> (FIM).
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">3. Anote a parada no </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>quadro 2</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">, com o </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Nº da peça</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> e o código do motivo.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">4. Voltou a produzir a mesma peça? Use o </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>próximo trecho da mesma linha</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">5. Troca de turno no meio da peça: o próximo operador usa o próximo trecho, com a chapa dele.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">6. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Peça pronta?</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> Escreva em </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>PRONTA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> o </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>turno que finalizou</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> (1, 2 ou 3). Não terminou? Deixe em branco e continue na próxima folha.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">7. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Mais de 4 trechos na mesma peça?</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> Continue na </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>linha de baixo</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">, com a mesma peça, e escreva em </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>CONTINUA A PEÇA Nº</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> o número da linha de cima. O turno em PRONTA vai só na última linha.</t>
-          </r>
-        </is>
-      </c>
-      <c r="B32" s="35" t="n"/>
-      <c r="C32" s="35" t="n"/>
-      <c r="D32" s="35" t="n"/>
-      <c r="E32" s="35" t="n"/>
-      <c r="F32" s="35" t="n"/>
-      <c r="G32" s="36" t="n"/>
-      <c r="H32" s="46" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+    <row r="32" ht="6" customHeight="1"/>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>COMO PREENCHER</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="n"/>
+      <c r="C33" s="38" t="n"/>
+      <c r="D33" s="38" t="n"/>
+      <c r="E33" s="38" t="n"/>
+      <c r="F33" s="38" t="n"/>
+      <c r="G33" s="37" t="n"/>
+      <c r="H33" s="21" t="inlineStr">
+        <is>
+          <t>CÓDIGOS DE PARADA (coluna MOTIVO)</t>
+        </is>
+      </c>
+      <c r="I33" s="38" t="n"/>
+      <c r="J33" s="38" t="n"/>
+      <c r="K33" s="38" t="n"/>
+      <c r="L33" s="37" t="n"/>
+      <c r="M33" s="21" t="inlineStr">
+        <is>
+          <t>EXEMPLO: MESA D61, 13:00 ÀS 17:00, PAROU 14:30–15:30</t>
+        </is>
+      </c>
+      <c r="N33" s="38" t="n"/>
+      <c r="O33" s="38" t="n"/>
+      <c r="P33" s="38" t="n"/>
+      <c r="Q33" s="38" t="n"/>
+      <c r="R33" s="38" t="n"/>
+      <c r="S33" s="37" t="n"/>
+    </row>
+    <row r="34" ht="13.5" customHeight="1">
+      <c r="A34" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>1. Uma linha = uma peça.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Começou peça nova? Linha nova.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G34" s="49" t="n"/>
+      <c r="H34" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
             </rPr>
             <t>1</t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Mecânica
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Mecânica</t>
+          </r>
+        </is>
+      </c>
+      <c r="J34" s="49" t="n"/>
+      <c r="K34" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>6</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Refeição</t>
+          </r>
+        </is>
+      </c>
+      <c r="L34" s="49" t="n"/>
+      <c r="M34" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Quadro 1 (peça 1):</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> MESA · D61 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · Pronta: 1</t>
+          </r>
+        </is>
+      </c>
+      <c r="S34" s="49" t="n"/>
+    </row>
+    <row r="35" ht="13.5" customHeight="1">
+      <c r="A35" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>2. Trecho = só produção.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Parou a máquina? Escreva o FIM do trecho.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
             </rPr>
             <t>2</t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Elétrica
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Elétrica</t>
+          </r>
+        </is>
+      </c>
+      <c r="J35" s="49" t="n"/>
+      <c r="K35" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>7</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Tyorei</t>
+          </r>
+        </is>
+      </c>
+      <c r="L35" s="49" t="n"/>
+      <c r="M35" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Quadro 2:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Nº da peça 1 · 14:30–15:30 · motivo 10 (troca de inserto)</t>
+          </r>
+        </is>
+      </c>
+      <c r="S35" s="49" t="n"/>
+    </row>
+    <row r="36" ht="13.5" customHeight="1">
+      <c r="A36" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>3. Anote a parada no quadro 2,</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> com o Nº da peça e o código do motivo.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
             </rPr>
             <t>3</t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Manutenção preventiva
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Manutenção preventiva</t>
+          </r>
+        </is>
+      </c>
+      <c r="J36" s="49" t="n"/>
+      <c r="K36" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>8</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Outros (descreva)</t>
+          </r>
+        </is>
+      </c>
+      <c r="L36" s="49" t="n"/>
+      <c r="M36" s="48" t="n"/>
+      <c r="S36" s="49" t="n"/>
+    </row>
+    <row r="37" ht="13.5" customHeight="1">
+      <c r="A37" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>4. Voltou a produzir a mesma peça?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Use o próximo trecho da mesma linha.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G37" s="49" t="n"/>
+      <c r="H37" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
             </rPr>
             <t>4</t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Troca de peça
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Troca de peça</t>
+          </r>
+        </is>
+      </c>
+      <c r="J37" s="49" t="n"/>
+      <c r="K37" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>9</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">  Set-up</t>
+          </r>
+        </is>
+      </c>
+      <c r="L37" s="49" t="n"/>
+      <c r="M37" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Certo:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> 3 h produzindo + 1 h parado = 4 h.</t>
+          </r>
+        </is>
+      </c>
+      <c r="S37" s="49" t="n"/>
+    </row>
+    <row r="38" ht="13.5" customHeight="1">
+      <c r="A38" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>5. Trocou o turno no meio da peça?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> O próximo operador usa o próximo trecho, com a chapa dele.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G38" s="49" t="n"/>
+      <c r="H38" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
             </rPr>
             <t>5</t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+              <sz val="9"/>
             </rPr>
             <t xml:space="preserve">  Falta de peça</t>
           </r>
         </is>
       </c>
-      <c r="I32" s="35" t="n"/>
-      <c r="J32" s="36" t="n"/>
-      <c r="K32" s="46" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t>6</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Refeição
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t>7</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Tyorei
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t>8</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Outros (descreva)
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t>9</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">  Set-up
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+      <c r="J38" s="49" t="n"/>
+      <c r="K38" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
             </rPr>
             <t>10</t>
           </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="12"/>
+              <sz val="9"/>
             </rPr>
             <t xml:space="preserve">  Ferramenta</t>
           </r>
         </is>
       </c>
-      <c r="L32" s="36" t="n"/>
-      <c r="M32" s="47" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Quadro 1 (peça 1): </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">MESA · D61 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · Pronta: 1
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Quadro 2: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Nº da peça 1 · 14:30–15:30 · motivo 10 (troca de inserto)
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Certo: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">3 h de produção + 1 h parada = 4 h.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Errado: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="11"/>
-            </rPr>
-            <t>um trecho 13:00–17:00 com a parada dentro dele (a hora parada conta duas vezes).</t>
-          </r>
-        </is>
-      </c>
-      <c r="N32" s="35" t="n"/>
-      <c r="O32" s="35" t="n"/>
-      <c r="P32" s="35" t="n"/>
-      <c r="Q32" s="35" t="n"/>
-      <c r="R32" s="35" t="n"/>
-      <c r="S32" s="36" t="n"/>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="43" t="n"/>
-      <c r="G33" s="44" t="n"/>
-      <c r="H33" s="43" t="n"/>
-      <c r="J33" s="44" t="n"/>
-      <c r="K33" s="43" t="n"/>
-      <c r="L33" s="44" t="n"/>
-      <c r="M33" s="43" t="n"/>
-      <c r="S33" s="44" t="n"/>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="43" t="n"/>
-      <c r="G34" s="44" t="n"/>
-      <c r="H34" s="43" t="n"/>
-      <c r="J34" s="44" t="n"/>
-      <c r="K34" s="43" t="n"/>
-      <c r="L34" s="44" t="n"/>
-      <c r="M34" s="43" t="n"/>
-      <c r="S34" s="44" t="n"/>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="43" t="n"/>
-      <c r="G35" s="44" t="n"/>
-      <c r="H35" s="43" t="n"/>
-      <c r="J35" s="44" t="n"/>
-      <c r="K35" s="43" t="n"/>
-      <c r="L35" s="44" t="n"/>
-      <c r="M35" s="43" t="n"/>
-      <c r="S35" s="44" t="n"/>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="43" t="n"/>
-      <c r="G36" s="44" t="n"/>
-      <c r="H36" s="43" t="n"/>
-      <c r="J36" s="44" t="n"/>
-      <c r="K36" s="43" t="n"/>
-      <c r="L36" s="44" t="n"/>
-      <c r="M36" s="43" t="n"/>
-      <c r="S36" s="44" t="n"/>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="43" t="n"/>
-      <c r="G37" s="44" t="n"/>
-      <c r="H37" s="43" t="n"/>
-      <c r="J37" s="44" t="n"/>
-      <c r="K37" s="43" t="n"/>
-      <c r="L37" s="44" t="n"/>
-      <c r="M37" s="43" t="n"/>
-      <c r="S37" s="44" t="n"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="39" t="n"/>
-      <c r="B38" s="40" t="n"/>
-      <c r="C38" s="40" t="n"/>
-      <c r="D38" s="40" t="n"/>
-      <c r="E38" s="40" t="n"/>
-      <c r="F38" s="40" t="n"/>
-      <c r="G38" s="41" t="n"/>
-      <c r="H38" s="39" t="n"/>
-      <c r="I38" s="40" t="n"/>
-      <c r="J38" s="41" t="n"/>
-      <c r="K38" s="39" t="n"/>
-      <c r="L38" s="41" t="n"/>
-      <c r="M38" s="39" t="n"/>
-      <c r="N38" s="40" t="n"/>
-      <c r="O38" s="40" t="n"/>
-      <c r="P38" s="40" t="n"/>
-      <c r="Q38" s="40" t="n"/>
-      <c r="R38" s="40" t="n"/>
-      <c r="S38" s="41" t="n"/>
-    </row>
+      <c r="L38" s="49" t="n"/>
+      <c r="M38" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Errado:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> um trecho só, 13:00–17:00, com a parada dentro dele.</t>
+          </r>
+        </is>
+      </c>
+      <c r="S38" s="49" t="n"/>
+    </row>
+    <row r="39" ht="13.5" customHeight="1">
+      <c r="A39" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>6. Peça pronta?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Escreva em PRONTA o turno (1, 2 ou 3). Não terminou? Deixe em branco.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G39" s="49" t="n"/>
+      <c r="H39" s="51" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>4 ou 9?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Outra peça igual = 4 · mudou de modelo = 9</t>
+          </r>
+        </is>
+      </c>
+      <c r="I39" s="52" t="n"/>
+      <c r="J39" s="52" t="n"/>
+      <c r="K39" s="52" t="n"/>
+      <c r="L39" s="53" t="n"/>
+      <c r="M39" s="48" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t>A hora parada contaria duas vezes.</t>
+          </r>
+        </is>
+      </c>
+      <c r="S39" s="49" t="n"/>
+    </row>
+    <row r="40" ht="13.5" customHeight="1">
+      <c r="A40" s="54" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>7. Mais de 4 trechos?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Siga na linha de baixo e escreva em CONTINUA o Nº da linha de cima.</t>
+          </r>
+        </is>
+      </c>
+      <c r="B40" s="55" t="n"/>
+      <c r="C40" s="55" t="n"/>
+      <c r="D40" s="55" t="n"/>
+      <c r="E40" s="55" t="n"/>
+      <c r="F40" s="55" t="n"/>
+      <c r="G40" s="56" t="n"/>
+      <c r="H40" s="57" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>1 ou 10?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> Inserto, fresa, broca = 10 · trocador = 1</t>
+          </r>
+        </is>
+      </c>
+      <c r="I40" s="58" t="n"/>
+      <c r="J40" s="58" t="n"/>
+      <c r="K40" s="58" t="n"/>
+      <c r="L40" s="59" t="n"/>
+      <c r="M40" s="54" t="n"/>
+      <c r="N40" s="55" t="n"/>
+      <c r="O40" s="55" t="n"/>
+      <c r="P40" s="55" t="n"/>
+      <c r="Q40" s="55" t="n"/>
+      <c r="R40" s="55" t="n"/>
+      <c r="S40" s="56" t="n"/>
+    </row>
+    <row r="41"/>
   </sheetData>
-  <mergeCells count="72">
+  <mergeCells count="94">
+    <mergeCell ref="M36:S36"/>
     <mergeCell ref="G21:H21"/>
+    <mergeCell ref="M33:S33"/>
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="M38:S38"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="L24:S24"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="L30:S30"/>
+    <mergeCell ref="L26:S26"/>
+    <mergeCell ref="L20:S20"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="L29:S29"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="L22:S22"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="L31:S31"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="R5:R6"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="L21:S21"/>
+    <mergeCell ref="H33:L33"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="L27:S27"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="K37:L37"/>
     <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="H36:J36"/>
     <mergeCell ref="E24:F24"/>
-    <mergeCell ref="K3:L3"/>
     <mergeCell ref="G27:H27"/>
     <mergeCell ref="N5:P5"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="L19:S19"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="L28:S28"/>
-    <mergeCell ref="H31:L31"/>
-    <mergeCell ref="A32:G38"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="M32:S38"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="A1:L2"/>
-    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="H40:L40"/>
+    <mergeCell ref="H39:L39"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="H37:J37"/>
     <mergeCell ref="E28:F28"/>
-    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="M37:S37"/>
     <mergeCell ref="G28:H28"/>
-    <mergeCell ref="L24:S24"/>
-    <mergeCell ref="L18:S18"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="K32:L38"/>
-    <mergeCell ref="L23:S23"/>
+    <mergeCell ref="M34:S34"/>
+    <mergeCell ref="Q2:S2"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="A5:A6"/>
-    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="L23:S23"/>
+    <mergeCell ref="A36:G36"/>
     <mergeCell ref="S5:S6"/>
-    <mergeCell ref="H32:J38"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="M39:S39"/>
+    <mergeCell ref="G30:H30"/>
     <mergeCell ref="G24:H24"/>
-    <mergeCell ref="L20:S20"/>
-    <mergeCell ref="L26:S26"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="L29:S29"/>
-    <mergeCell ref="E27:F27"/>
     <mergeCell ref="L25:S25"/>
-    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="M35:S35"/>
+    <mergeCell ref="H35:J35"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="L22:S22"/>
     <mergeCell ref="G26:H26"/>
-    <mergeCell ref="A17:H17"/>
     <mergeCell ref="D5:D6"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="A4:H4"/>
     <mergeCell ref="G29:H29"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="R5:R6"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="I17:S17"/>
-    <mergeCell ref="M31:S31"/>
     <mergeCell ref="I4:S4"/>
     <mergeCell ref="E5:G5"/>
-    <mergeCell ref="K5:M5"/>
     <mergeCell ref="E25:F25"/>
+    <mergeCell ref="K38:L38"/>
     <mergeCell ref="G25:H25"/>
-    <mergeCell ref="L21:S21"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="L27:S27"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="M40:S40"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="I19:S19"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="K3:L3"/>
     <mergeCell ref="C5:C6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
Excel: ajustar em uma página explícito
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019Px7p5mhzWYWbE6aV5W89g
</commit_message>
<xml_diff>
--- a/docs/folha-modelo/diario-de-bordo.xlsx
+++ b/docs/folha-modelo/diario-de-bordo.xlsx
@@ -189,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -416,11 +416,35 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -561,6 +585,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1837,7 +1870,7 @@
       <c r="S33" s="37" t="n"/>
     </row>
     <row r="34" ht="13.5" customHeight="1">
-      <c r="A34" s="48" t="inlineStr">
+      <c r="A34" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1857,7 +1890,7 @@
         </is>
       </c>
       <c r="G34" s="49" t="n"/>
-      <c r="H34" s="48" t="inlineStr">
+      <c r="H34" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1877,7 +1910,7 @@
         </is>
       </c>
       <c r="J34" s="49" t="n"/>
-      <c r="K34" s="48" t="inlineStr">
+      <c r="K34" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1897,7 +1930,7 @@
         </is>
       </c>
       <c r="L34" s="49" t="n"/>
-      <c r="M34" s="48" t="inlineStr">
+      <c r="M34" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1919,7 +1952,7 @@
       <c r="S34" s="49" t="n"/>
     </row>
     <row r="35" ht="13.5" customHeight="1">
-      <c r="A35" s="48" t="inlineStr">
+      <c r="A35" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1939,7 +1972,7 @@
         </is>
       </c>
       <c r="G35" s="49" t="n"/>
-      <c r="H35" s="48" t="inlineStr">
+      <c r="H35" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1959,7 +1992,7 @@
         </is>
       </c>
       <c r="J35" s="49" t="n"/>
-      <c r="K35" s="48" t="inlineStr">
+      <c r="K35" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1979,7 +2012,7 @@
         </is>
       </c>
       <c r="L35" s="49" t="n"/>
-      <c r="M35" s="48" t="inlineStr">
+      <c r="M35" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2001,7 +2034,7 @@
       <c r="S35" s="49" t="n"/>
     </row>
     <row r="36" ht="13.5" customHeight="1">
-      <c r="A36" s="48" t="inlineStr">
+      <c r="A36" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2021,7 +2054,7 @@
         </is>
       </c>
       <c r="G36" s="49" t="n"/>
-      <c r="H36" s="48" t="inlineStr">
+      <c r="H36" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2041,7 +2074,7 @@
         </is>
       </c>
       <c r="J36" s="49" t="n"/>
-      <c r="K36" s="48" t="inlineStr">
+      <c r="K36" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2061,11 +2094,11 @@
         </is>
       </c>
       <c r="L36" s="49" t="n"/>
-      <c r="M36" s="48" t="n"/>
+      <c r="M36" s="60" t="n"/>
       <c r="S36" s="49" t="n"/>
     </row>
     <row r="37" ht="13.5" customHeight="1">
-      <c r="A37" s="48" t="inlineStr">
+      <c r="A37" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2085,7 +2118,7 @@
         </is>
       </c>
       <c r="G37" s="49" t="n"/>
-      <c r="H37" s="48" t="inlineStr">
+      <c r="H37" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2105,7 +2138,7 @@
         </is>
       </c>
       <c r="J37" s="49" t="n"/>
-      <c r="K37" s="48" t="inlineStr">
+      <c r="K37" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2125,7 +2158,7 @@
         </is>
       </c>
       <c r="L37" s="49" t="n"/>
-      <c r="M37" s="48" t="inlineStr">
+      <c r="M37" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2147,7 +2180,7 @@
       <c r="S37" s="49" t="n"/>
     </row>
     <row r="38" ht="13.5" customHeight="1">
-      <c r="A38" s="48" t="inlineStr">
+      <c r="A38" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2167,11 +2200,11 @@
         </is>
       </c>
       <c r="G38" s="49" t="n"/>
-      <c r="H38" s="50" t="n"/>
+      <c r="H38" s="61" t="n"/>
       <c r="J38" s="49" t="n"/>
-      <c r="K38" s="50" t="n"/>
+      <c r="K38" s="61" t="n"/>
       <c r="L38" s="49" t="n"/>
-      <c r="M38" s="48" t="inlineStr">
+      <c r="M38" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2193,7 +2226,7 @@
       <c r="S38" s="49" t="n"/>
     </row>
     <row r="39" ht="13.5" customHeight="1">
-      <c r="A39" s="48" t="inlineStr">
+      <c r="A39" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2213,7 +2246,7 @@
         </is>
       </c>
       <c r="G39" s="49" t="n"/>
-      <c r="H39" s="51" t="inlineStr">
+      <c r="H39" s="62" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2232,11 +2265,11 @@
           </r>
         </is>
       </c>
-      <c r="I39" s="52" t="n"/>
-      <c r="J39" s="52" t="n"/>
-      <c r="K39" s="52" t="n"/>
-      <c r="L39" s="53" t="n"/>
-      <c r="M39" s="48" t="inlineStr">
+      <c r="I39" s="63" t="n"/>
+      <c r="J39" s="63" t="n"/>
+      <c r="K39" s="63" t="n"/>
+      <c r="L39" s="64" t="n"/>
+      <c r="M39" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2275,7 +2308,7 @@
       <c r="E40" s="55" t="n"/>
       <c r="F40" s="55" t="n"/>
       <c r="G40" s="56" t="n"/>
-      <c r="H40" s="57" t="inlineStr">
+      <c r="H40" s="54" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2294,10 +2327,10 @@
           </r>
         </is>
       </c>
-      <c r="I40" s="58" t="n"/>
-      <c r="J40" s="58" t="n"/>
-      <c r="K40" s="58" t="n"/>
-      <c r="L40" s="59" t="n"/>
+      <c r="I40" s="55" t="n"/>
+      <c r="J40" s="55" t="n"/>
+      <c r="K40" s="55" t="n"/>
+      <c r="L40" s="56" t="n"/>
       <c r="M40" s="54" t="n"/>
       <c r="N40" s="55" t="n"/>
       <c r="O40" s="55" t="n"/>
@@ -2306,107 +2339,106 @@
       <c r="R40" s="55" t="n"/>
       <c r="S40" s="56" t="n"/>
     </row>
-    <row r="41"/>
   </sheetData>
   <mergeCells count="94">
     <mergeCell ref="M36:S36"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="M33:S33"/>
-    <mergeCell ref="K3:L3"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="E23:F23"/>
-    <mergeCell ref="A38:G38"/>
     <mergeCell ref="G23:H23"/>
-    <mergeCell ref="M38:S38"/>
     <mergeCell ref="K35:L35"/>
-    <mergeCell ref="M2:N2"/>
     <mergeCell ref="N3:O3"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="A40:G40"/>
-    <mergeCell ref="E29:F29"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="A1:L2"/>
     <mergeCell ref="O1:P1"/>
     <mergeCell ref="L24:S24"/>
+    <mergeCell ref="L26:S26"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="L27:S27"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="L28:S28"/>
+    <mergeCell ref="H40:L40"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="M34:S34"/>
+    <mergeCell ref="L23:S23"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="M39:S39"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="H35:J35"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="M40:S40"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="I19:S19"/>
+    <mergeCell ref="M37:S37"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="M38:S38"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="E29:F29"/>
     <mergeCell ref="I20:K20"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="E31:F31"/>
     <mergeCell ref="L30:S30"/>
-    <mergeCell ref="L26:S26"/>
     <mergeCell ref="L20:S20"/>
-    <mergeCell ref="H5:J5"/>
     <mergeCell ref="L29:S29"/>
-    <mergeCell ref="E27:F27"/>
     <mergeCell ref="C3:H3"/>
     <mergeCell ref="L22:S22"/>
-    <mergeCell ref="A37:G37"/>
-    <mergeCell ref="H38:J38"/>
     <mergeCell ref="L31:S31"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="G20:H20"/>
     <mergeCell ref="R5:R6"/>
-    <mergeCell ref="K5:M5"/>
     <mergeCell ref="L21:S21"/>
     <mergeCell ref="H33:L33"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="L27:S27"/>
     <mergeCell ref="A19:H19"/>
-    <mergeCell ref="G22:H22"/>
     <mergeCell ref="H34:J34"/>
-    <mergeCell ref="K37:L37"/>
-    <mergeCell ref="Q5:Q6"/>
     <mergeCell ref="K34:L34"/>
     <mergeCell ref="H36:J36"/>
     <mergeCell ref="E24:F24"/>
     <mergeCell ref="G27:H27"/>
     <mergeCell ref="N5:P5"/>
-    <mergeCell ref="M1:N1"/>
     <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="L28:S28"/>
     <mergeCell ref="K36:L36"/>
-    <mergeCell ref="H40:L40"/>
     <mergeCell ref="H39:L39"/>
-    <mergeCell ref="A34:G34"/>
     <mergeCell ref="H37:J37"/>
     <mergeCell ref="E28:F28"/>
-    <mergeCell ref="M37:S37"/>
     <mergeCell ref="G28:H28"/>
-    <mergeCell ref="M34:S34"/>
     <mergeCell ref="Q2:S2"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="A5:A6"/>
-    <mergeCell ref="L23:S23"/>
-    <mergeCell ref="A36:G36"/>
     <mergeCell ref="S5:S6"/>
     <mergeCell ref="E30:F30"/>
-    <mergeCell ref="M39:S39"/>
     <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G24:H24"/>
     <mergeCell ref="L25:S25"/>
     <mergeCell ref="M35:S35"/>
-    <mergeCell ref="H35:J35"/>
-    <mergeCell ref="E26:F26"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="G26:H26"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="Q3:S3"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="G29:H29"/>
     <mergeCell ref="I4:S4"/>
     <mergeCell ref="E5:G5"/>
-    <mergeCell ref="E25:F25"/>
     <mergeCell ref="K38:L38"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="M40:S40"/>
     <mergeCell ref="G31:H31"/>
-    <mergeCell ref="I19:S19"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="E21:F21"/>
-    <mergeCell ref="C5:C6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0" footer="0"/>
-  <pageSetup orientation="landscape" paperSize="9" scale="77"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="77" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -3327,7 +3359,7 @@
       <c r="S33" s="37" t="n"/>
     </row>
     <row r="34" ht="13.5" customHeight="1">
-      <c r="A34" s="48" t="inlineStr">
+      <c r="A34" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3347,7 +3379,7 @@
         </is>
       </c>
       <c r="G34" s="49" t="n"/>
-      <c r="H34" s="48" t="inlineStr">
+      <c r="H34" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3367,7 +3399,7 @@
         </is>
       </c>
       <c r="J34" s="49" t="n"/>
-      <c r="K34" s="48" t="inlineStr">
+      <c r="K34" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3387,7 +3419,7 @@
         </is>
       </c>
       <c r="L34" s="49" t="n"/>
-      <c r="M34" s="48" t="inlineStr">
+      <c r="M34" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3409,7 +3441,7 @@
       <c r="S34" s="49" t="n"/>
     </row>
     <row r="35" ht="13.5" customHeight="1">
-      <c r="A35" s="48" t="inlineStr">
+      <c r="A35" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3429,7 +3461,7 @@
         </is>
       </c>
       <c r="G35" s="49" t="n"/>
-      <c r="H35" s="48" t="inlineStr">
+      <c r="H35" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3449,7 +3481,7 @@
         </is>
       </c>
       <c r="J35" s="49" t="n"/>
-      <c r="K35" s="48" t="inlineStr">
+      <c r="K35" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3469,7 +3501,7 @@
         </is>
       </c>
       <c r="L35" s="49" t="n"/>
-      <c r="M35" s="48" t="inlineStr">
+      <c r="M35" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3491,7 +3523,7 @@
       <c r="S35" s="49" t="n"/>
     </row>
     <row r="36" ht="13.5" customHeight="1">
-      <c r="A36" s="48" t="inlineStr">
+      <c r="A36" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3511,7 +3543,7 @@
         </is>
       </c>
       <c r="G36" s="49" t="n"/>
-      <c r="H36" s="48" t="inlineStr">
+      <c r="H36" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3531,7 +3563,7 @@
         </is>
       </c>
       <c r="J36" s="49" t="n"/>
-      <c r="K36" s="48" t="inlineStr">
+      <c r="K36" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3551,11 +3583,11 @@
         </is>
       </c>
       <c r="L36" s="49" t="n"/>
-      <c r="M36" s="48" t="n"/>
+      <c r="M36" s="60" t="n"/>
       <c r="S36" s="49" t="n"/>
     </row>
     <row r="37" ht="13.5" customHeight="1">
-      <c r="A37" s="48" t="inlineStr">
+      <c r="A37" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3575,7 +3607,7 @@
         </is>
       </c>
       <c r="G37" s="49" t="n"/>
-      <c r="H37" s="48" t="inlineStr">
+      <c r="H37" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3595,7 +3627,7 @@
         </is>
       </c>
       <c r="J37" s="49" t="n"/>
-      <c r="K37" s="48" t="inlineStr">
+      <c r="K37" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3615,7 +3647,7 @@
         </is>
       </c>
       <c r="L37" s="49" t="n"/>
-      <c r="M37" s="48" t="inlineStr">
+      <c r="M37" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3637,7 +3669,7 @@
       <c r="S37" s="49" t="n"/>
     </row>
     <row r="38" ht="13.5" customHeight="1">
-      <c r="A38" s="48" t="inlineStr">
+      <c r="A38" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3657,7 +3689,7 @@
         </is>
       </c>
       <c r="G38" s="49" t="n"/>
-      <c r="H38" s="48" t="inlineStr">
+      <c r="H38" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3677,7 +3709,7 @@
         </is>
       </c>
       <c r="J38" s="49" t="n"/>
-      <c r="K38" s="48" t="inlineStr">
+      <c r="K38" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3697,7 +3729,7 @@
         </is>
       </c>
       <c r="L38" s="49" t="n"/>
-      <c r="M38" s="48" t="inlineStr">
+      <c r="M38" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3719,7 +3751,7 @@
       <c r="S38" s="49" t="n"/>
     </row>
     <row r="39" ht="13.5" customHeight="1">
-      <c r="A39" s="48" t="inlineStr">
+      <c r="A39" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3739,7 +3771,7 @@
         </is>
       </c>
       <c r="G39" s="49" t="n"/>
-      <c r="H39" s="51" t="inlineStr">
+      <c r="H39" s="62" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3758,11 +3790,11 @@
           </r>
         </is>
       </c>
-      <c r="I39" s="52" t="n"/>
-      <c r="J39" s="52" t="n"/>
-      <c r="K39" s="52" t="n"/>
-      <c r="L39" s="53" t="n"/>
-      <c r="M39" s="48" t="inlineStr">
+      <c r="I39" s="63" t="n"/>
+      <c r="J39" s="63" t="n"/>
+      <c r="K39" s="63" t="n"/>
+      <c r="L39" s="64" t="n"/>
+      <c r="M39" s="60" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3801,7 +3833,7 @@
       <c r="E40" s="55" t="n"/>
       <c r="F40" s="55" t="n"/>
       <c r="G40" s="56" t="n"/>
-      <c r="H40" s="57" t="inlineStr">
+      <c r="H40" s="54" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3820,10 +3852,10 @@
           </r>
         </is>
       </c>
-      <c r="I40" s="58" t="n"/>
-      <c r="J40" s="58" t="n"/>
-      <c r="K40" s="58" t="n"/>
-      <c r="L40" s="59" t="n"/>
+      <c r="I40" s="55" t="n"/>
+      <c r="J40" s="55" t="n"/>
+      <c r="K40" s="55" t="n"/>
+      <c r="L40" s="56" t="n"/>
       <c r="M40" s="54" t="n"/>
       <c r="N40" s="55" t="n"/>
       <c r="O40" s="55" t="n"/>
@@ -3832,7 +3864,6 @@
       <c r="R40" s="55" t="n"/>
       <c r="S40" s="56" t="n"/>
     </row>
-    <row r="41"/>
   </sheetData>
   <mergeCells count="94">
     <mergeCell ref="M36:S36"/>
@@ -3840,99 +3871,99 @@
     <mergeCell ref="M33:S33"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="E23:F23"/>
-    <mergeCell ref="A38:G38"/>
     <mergeCell ref="G23:H23"/>
-    <mergeCell ref="M38:S38"/>
     <mergeCell ref="K35:L35"/>
-    <mergeCell ref="M2:N2"/>
     <mergeCell ref="N3:O3"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="A40:G40"/>
-    <mergeCell ref="E29:F29"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="A1:L2"/>
     <mergeCell ref="O1:P1"/>
     <mergeCell ref="L24:S24"/>
+    <mergeCell ref="L26:S26"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="L27:S27"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="L28:S28"/>
+    <mergeCell ref="H40:L40"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="M34:S34"/>
+    <mergeCell ref="L23:S23"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="M39:S39"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="H35:J35"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="M40:S40"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="I19:S19"/>
+    <mergeCell ref="M37:S37"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="M38:S38"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="E29:F29"/>
     <mergeCell ref="I20:K20"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="E31:F31"/>
     <mergeCell ref="L30:S30"/>
-    <mergeCell ref="L26:S26"/>
     <mergeCell ref="L20:S20"/>
-    <mergeCell ref="H5:J5"/>
     <mergeCell ref="L29:S29"/>
-    <mergeCell ref="E27:F27"/>
     <mergeCell ref="C3:H3"/>
     <mergeCell ref="L22:S22"/>
-    <mergeCell ref="A37:G37"/>
-    <mergeCell ref="H38:J38"/>
     <mergeCell ref="L31:S31"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="G20:H20"/>
     <mergeCell ref="R5:R6"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="K5:M5"/>
     <mergeCell ref="L21:S21"/>
     <mergeCell ref="H33:L33"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="L27:S27"/>
     <mergeCell ref="A19:H19"/>
-    <mergeCell ref="G22:H22"/>
     <mergeCell ref="H34:J34"/>
-    <mergeCell ref="K37:L37"/>
-    <mergeCell ref="Q5:Q6"/>
     <mergeCell ref="K34:L34"/>
     <mergeCell ref="H36:J36"/>
     <mergeCell ref="E24:F24"/>
     <mergeCell ref="G27:H27"/>
     <mergeCell ref="N5:P5"/>
-    <mergeCell ref="M1:N1"/>
     <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="L28:S28"/>
     <mergeCell ref="K36:L36"/>
-    <mergeCell ref="H40:L40"/>
     <mergeCell ref="H39:L39"/>
-    <mergeCell ref="A34:G34"/>
     <mergeCell ref="H37:J37"/>
     <mergeCell ref="E28:F28"/>
-    <mergeCell ref="M37:S37"/>
     <mergeCell ref="G28:H28"/>
-    <mergeCell ref="M34:S34"/>
     <mergeCell ref="Q2:S2"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="A5:A6"/>
-    <mergeCell ref="L23:S23"/>
-    <mergeCell ref="A36:G36"/>
     <mergeCell ref="S5:S6"/>
     <mergeCell ref="E30:F30"/>
-    <mergeCell ref="M39:S39"/>
     <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G24:H24"/>
     <mergeCell ref="L25:S25"/>
     <mergeCell ref="M35:S35"/>
-    <mergeCell ref="H35:J35"/>
-    <mergeCell ref="E26:F26"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="G26:H26"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="Q3:S3"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="G29:H29"/>
     <mergeCell ref="I4:S4"/>
     <mergeCell ref="E5:G5"/>
-    <mergeCell ref="E25:F25"/>
     <mergeCell ref="K38:L38"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="M40:S40"/>
     <mergeCell ref="G31:H31"/>
-    <mergeCell ref="I19:S19"/>
     <mergeCell ref="A33:G33"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="E21:F21"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0" footer="0"/>
-  <pageSetup orientation="landscape" paperSize="9" scale="77"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="77" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -6142,6 +6173,6 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0" footer="0"/>
-  <pageSetup orientation="portrait" paperSize="8" scale="87"/>
+  <pageSetup orientation="portrait" paperSize="8" scale="87" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>